<commit_message>
Update: Added documentation for two functions.
I added documentation for the first two function in the program.  This will make sure the program works as intended.
</commit_message>
<xml_diff>
--- a/Test-Cases/Testing-Script-Records.xlsx
+++ b/Test-Cases/Testing-Script-Records.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30520"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4872d23a9318b819/Documents/GitHub/Ophelias-Oasis/Test-Cases/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexahope/Documents/GitHub/Ophelias-Oasis/Test-Cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="383" documentId="8_{1BAE7848-AFB0-FA4A-AF2B-72F0321F99E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A3A047F-CC89-41C1-8FB0-7FF4937B7C31}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC38B1CA-139B-9745-9A4A-4FBE3F148D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" firstSheet="1" activeTab="1" xr2:uid="{32C5AFC3-1601-AE47-BE56-3877807D3FAA}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19700" windowHeight="21600" firstSheet="1" activeTab="1" xr2:uid="{32C5AFC3-1601-AE47-BE56-3877807D3FAA}"/>
   </bookViews>
   <sheets>
     <sheet name="Test-Documentation" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="225">
   <si>
     <t>Transaction ID:</t>
   </si>
@@ -667,13 +667,61 @@
   </si>
   <si>
     <t>addReportedReservationPricing</t>
+  </si>
+  <si>
+    <t>Sally, Ben, Keith, Harvey, Sam, Drake, Eithan, Lee, Nick, Jack</t>
+  </si>
+  <si>
+    <t>Double, Double, Double, Double, Double, Double, Double, Double, Double, Double.</t>
+  </si>
+  <si>
+    <t>20000, 40000, 31000, 40000, 60000, 700000, 21000, 23000, 25999, 21099</t>
+  </si>
+  <si>
+    <t>"Changed due to broken leg.", "Changed due to a updated status of disability.", "Change due to more time being required to develop platform for users.", "Changed due to a lack of data support claim.", "Change due to problems in social organization within their workforce.", "The ability for a person status to change is due to issues in the local goverment.  This person accomdation has change due to the power shifts in the local goverment.", "Their is not enough resources to provide this accomdation for this person", "Their is not enough time to provide resources for this person", "Their is not enough memory in the computer to provide accomdation for this person.", "Their is not witness to account for this person disability."</t>
+  </si>
+  <si>
+    <t>Bool, Bool, Bool, Bool, Bool, Bool, Bool, Bool, Bool, Bool</t>
+  </si>
+  <si>
+    <t>True, True, True, True, True, True, True, True, True, True</t>
+  </si>
+  <si>
+    <t>Used for understanding and printing report for the users.  This is just to describe the report for the users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The first parameter describes the name of the function.  It is used to understand the functions use cases.  </t>
+  </si>
+  <si>
+    <t>The function outputs the description for the selected function.</t>
+  </si>
+  <si>
+    <t>The function is used for describing the accomdation a person receives.  This process is used to understand what accomdation a person receives and how they will impact their stay at Ophelias-Oasis.</t>
+  </si>
+  <si>
+    <t>The input parameters states the name of the accomdation and the change in budget as well as the state of the change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The output state whiether the change for the output has been completed successful.  This is require to make sure the change works as intended.  </t>
+  </si>
+  <si>
+    <t>"1: Changed accomdation report for saterday., 2: Change the problems in the accomdation report., 3: Change problems due to weightloss.", "1: Issues in health addressed, 2: Issues in in physciology in and issues in time management.", "1: Issues in process accomdations that prevent user needs from being addressed.", "1: Change accomdation report to accomdate for changing or rising cost of price.", "1: Change accomdation to account for problems in process of this software.", "1: Change issues in the ecomony., 2: Change issues related to the size of the company., 3: Problems in the software the prevent the accodations from loading and prevent them from working as intended.", "1: Making sure to allow the functions to work as intended so the program will work, 2: Make sure problems in the code are able to be debugged.", "1: The process loading accomdation is blocked, 2: The process of changing accomdation is blocked, 3: The process of seeing accomdation is blocked, 4: The process of seeing issues in the goverments.", "1: Problems in work cited for accomdations, 2: Noticed issues in problems for the broadcasting of data in the software., 3: Issues in the software that prevent it from functions., 4: Issues that prevent problems from loading accomdation in the software.", "1: The process of accounting for changes in accomdations."</t>
+  </si>
+  <si>
+    <t>The function is used for describing the history of reports.  This reports is process will allow the program to work as intended and report a history of accomdations.</t>
+  </si>
+  <si>
+    <t>The parameters of the function is the name which identity which person you are pulling up a full report of the person for.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The output is a string returning the complete history of the person.  This will allow for the user to understand how their accomdation and needs changes over time.  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1064,20 +1112,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4773A701-89D4-DA4B-93FB-4CFE88602652}">
   <dimension ref="A1:H51"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="16.125" customWidth="1"/>
-    <col min="3" max="3" width="17.875" customWidth="1"/>
-    <col min="4" max="4" width="18.625" customWidth="1"/>
-    <col min="5" max="5" width="16.625" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="33.125" customWidth="1"/>
-    <col min="8" max="8" width="27.625" customWidth="1"/>
-    <col min="9" max="9" width="26.875" customWidth="1"/>
+    <col min="7" max="7" width="33.1640625" customWidth="1"/>
+    <col min="8" max="8" width="27.6640625" customWidth="1"/>
+    <col min="9" max="9" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1100,252 +1148,252 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:1">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:1">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:1">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:1">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:1">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:1">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:1">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:1">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:1">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:1">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:1">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:1">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:1">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:1">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:1">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:1">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:1">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:1">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:1">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:1">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:1">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:1">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>56</v>
       </c>
@@ -1358,14 +1406,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44E41573-350E-4D19-A26B-D0AE87797D6F}">
   <dimension ref="A1:BR62"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="20.625" customWidth="1"/>
-    <col min="9" max="9" width="47.875" customWidth="1"/>
-    <col min="10" max="10" width="58.75" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="47.83203125" customWidth="1"/>
+    <col min="10" max="10" width="58.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:70">
+    <row r="1" spans="1:70" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
         <v>57</v>
       </c>
@@ -1448,7 +1496,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:70">
+    <row r="2" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>84</v>
       </c>
@@ -1470,8 +1518,17 @@
       <c r="BI2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="3" spans="1:70">
+      <c r="BL2" t="s">
+        <v>215</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>216</v>
+      </c>
+      <c r="BR2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="3" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>89</v>
       </c>
@@ -1479,10 +1536,43 @@
         <v>90</v>
       </c>
       <c r="E3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:70">
+        <v>3</v>
+      </c>
+      <c r="H3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J3" t="s">
+        <v>209</v>
+      </c>
+      <c r="M3" t="s">
+        <v>210</v>
+      </c>
+      <c r="O3" t="s">
+        <v>211</v>
+      </c>
+      <c r="R3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T3" t="s">
+        <v>212</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>214</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>218</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>219</v>
+      </c>
+      <c r="BR3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="4" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>91</v>
       </c>
@@ -1492,8 +1582,29 @@
       <c r="E4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:70">
+      <c r="H4" t="s">
+        <v>86</v>
+      </c>
+      <c r="J4" t="s">
+        <v>209</v>
+      </c>
+      <c r="BF4" t="s">
+        <v>86</v>
+      </c>
+      <c r="BI4" t="s">
+        <v>221</v>
+      </c>
+      <c r="BL4" t="s">
+        <v>222</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>223</v>
+      </c>
+      <c r="BR4" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="5" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>93</v>
       </c>
@@ -1504,7 +1615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:70">
+    <row r="6" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -1515,7 +1626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:70">
+    <row r="7" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -1526,7 +1637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:70">
+    <row r="8" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -1537,7 +1648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:70">
+    <row r="9" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>101</v>
       </c>
@@ -1548,7 +1659,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:70">
+    <row r="10" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>103</v>
       </c>
@@ -1559,7 +1670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:70">
+    <row r="11" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>105</v>
       </c>
@@ -1570,7 +1681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:70">
+    <row r="12" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>107</v>
       </c>
@@ -1581,7 +1692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:70">
+    <row r="13" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>109</v>
       </c>
@@ -1592,7 +1703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:70">
+    <row r="14" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>111</v>
       </c>
@@ -1603,7 +1714,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:70">
+    <row r="15" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>113</v>
       </c>
@@ -1614,7 +1725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:70">
+    <row r="16" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>115</v>
       </c>
@@ -1625,7 +1736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>117</v>
       </c>
@@ -1636,7 +1747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>119</v>
       </c>
@@ -1647,7 +1758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>121</v>
       </c>
@@ -1658,7 +1769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>123</v>
       </c>
@@ -1669,7 +1780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>125</v>
       </c>
@@ -1680,7 +1791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>127</v>
       </c>
@@ -1691,7 +1802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>129</v>
       </c>
@@ -1702,7 +1813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>131</v>
       </c>
@@ -1713,7 +1824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>133</v>
       </c>
@@ -1724,7 +1835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>135</v>
       </c>
@@ -1735,7 +1846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>137</v>
       </c>
@@ -1746,7 +1857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>139</v>
       </c>
@@ -1757,7 +1868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>141</v>
       </c>
@@ -1768,7 +1879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>143</v>
       </c>
@@ -1779,7 +1890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>145</v>
       </c>
@@ -1790,7 +1901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>147</v>
       </c>
@@ -1801,7 +1912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>149</v>
       </c>
@@ -1812,7 +1923,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>151</v>
       </c>
@@ -1823,7 +1934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>153</v>
       </c>
@@ -1834,7 +1945,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>155</v>
       </c>
@@ -1845,7 +1956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>157</v>
       </c>
@@ -1856,7 +1967,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>159</v>
       </c>
@@ -1867,7 +1978,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>161</v>
       </c>
@@ -1878,7 +1989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>163</v>
       </c>
@@ -1889,7 +2000,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>165</v>
       </c>
@@ -1900,7 +2011,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>167</v>
       </c>
@@ -1911,7 +2022,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>169</v>
       </c>
@@ -1922,7 +2033,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>171</v>
       </c>
@@ -1933,7 +2044,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>173</v>
       </c>
@@ -1944,7 +2055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>175</v>
       </c>
@@ -1955,7 +2066,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>177</v>
       </c>
@@ -1966,7 +2077,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>179</v>
       </c>
@@ -1977,7 +2088,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>181</v>
       </c>
@@ -1988,7 +2099,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>183</v>
       </c>
@@ -1999,7 +2110,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>185</v>
       </c>
@@ -2010,7 +2121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>187</v>
       </c>
@@ -2021,7 +2132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>189</v>
       </c>
@@ -2032,7 +2143,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>191</v>
       </c>
@@ -2043,7 +2154,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>193</v>
       </c>
@@ -2054,7 +2165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>195</v>
       </c>
@@ -2065,7 +2176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>197</v>
       </c>
@@ -2076,7 +2187,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>199</v>
       </c>
@@ -2087,7 +2198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>201</v>
       </c>
@@ -2098,7 +2209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>203</v>
       </c>
@@ -2109,7 +2220,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>205</v>
       </c>
@@ -2120,7 +2231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>207</v>
       </c>

</xml_diff>

<commit_message>
Update: Added the first 15 test entries.
I added the first 15 test entries for the program.  This will make sure the program will work as intended.  This will also make sure to test it user the known data for the project.  This makes sure the project works as intended.
</commit_message>
<xml_diff>
--- a/Test-Cases/Testing-Script-Records.xlsx
+++ b/Test-Cases/Testing-Script-Records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexahope/Documents/GitHub/Ophelias-Oasis/Test-Cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96020CC2-2A9E-E349-A5E5-281E850170E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE61DDA-9E21-4B45-8BDA-E4D5599A02D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" firstSheet="1" activeTab="1" xr2:uid="{32C5AFC3-1601-AE47-BE56-3877807D3FAA}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="278">
   <si>
     <t>Transaction ID:</t>
   </si>
@@ -745,13 +745,142 @@
   </si>
   <si>
     <t>The function outputs a help menu describing how the program works.  It used for documenting the program and allow for users to understand how to user the program.  This allows for the user to overall understand the user case for the program.  It will allow for them to interface for the program as well.</t>
+  </si>
+  <si>
+    <t>"~/", "/", "~/.Emu-Backup", "~/.Emu-Root-Backup", "~/Downloads/Emu-Backup", "Emu-Backup", "Emu-Root-Backup", "EmuBackup", "EmuRootBackup", "~/Local/EmuBackup"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function allows for setting the local location of the backup.  This backup allow for the program to take local backups of the system which allows for it to work as intended.  </t>
+  </si>
+  <si>
+    <t>The parameters are the name of the local backup location.  This allows for the function to set a local backup locals which is a requirement of the program for it to work as intended.</t>
+  </si>
+  <si>
+    <t>The output of this program is true if the back up works as inteded.  It return false if the backup does not work as intended.  Hence, this does not pass the test as we are requiring the program to work.</t>
+  </si>
+  <si>
+    <t>The function test if the program is working as intended.  The software should be able to delete the backups created at each of those location.  If it is not able to it will return a false.  This means the program has not worked as itnended.  However, we need to stil have other functionality in the program testing those files have been created and distroyed in later iteration of this testing program.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The parameter shows the location of the backup in the system memory.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function outputs true when the backup has gone as intended.  The function outputs false when the function has failed to backup.  We want the function to output true for the backup task to work as intended.  This will make sure the program works and passes all the requirements.  </t>
+  </si>
+  <si>
+    <t>Sally, Bem, Keith, Harvey, Sam, Drake, Eithan, Lee, Nick, Jack</t>
+  </si>
+  <si>
+    <t>Int, Int, Int, Int, Int, Int, Int, Int, Int, Int</t>
+  </si>
+  <si>
+    <t>200, 2101, 3020, 1002, 1023, 2028, 203, 209, 2731, 2804</t>
+  </si>
+  <si>
+    <t>Int[3], Int[3], Int[3], Int[3], Int[3], Int[3], Int[3], Int[3], Int[3], Int[3]</t>
+  </si>
+  <si>
+    <t>[3, 21, 2026], [4, 21, 2010], [4, 28, 2024], [5, 11, 2023], [8, 13, 2022], [7, 15, 2025], [3, 23, 2024], [8, 27, 2026], [11, 23, 2026], [12, 29, 2026]</t>
+  </si>
+  <si>
+    <t>This function allows for creating a booking entry.  The system is testing to make sure you have made a booking entry as intended by the programmers of the program.</t>
+  </si>
+  <si>
+    <t>The parameters include, the users name, the room they are booking, and, the date of the transaction.  The name is the name of the users who is working on the project.  The data of the transaction is the data in which the transaction took place.  The room number is the number of the room the users is trying to book.</t>
+  </si>
+  <si>
+    <t>The function outputs true when the function has been able to create the booking entry successful.  The function outputs false when the function has not been able to output the booking entry sucessfully.  This allows for the users to know if the transaction has occured successfully or not.</t>
+  </si>
+  <si>
+    <t>The function allows for deleting a bookign entry.  It will allow the users  to delete the local booking entry to make sure the transaction works as intended.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The entries include the users name, date of transaction, and, the room.  The name is the name of the target users.  The date of the transaction is the date the transaction occur.  The room numbers is the number of the room we are targeting.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function true when the booking entry has successful been deleted.  The function outputs false when the booking entry has not been successful deleted.  This allows for the program to test if the program is able to delete booking entries successful as intended. </t>
+  </si>
+  <si>
+    <t>Int[3], Int[3], Int[3], Int[3], Int[3], Int[3], Int[3], Int[3]</t>
+  </si>
+  <si>
+    <t>[4, 9, 2000], [4, 8, 2010], [3, 2, 2029], [2, 3, 2020], [2, 3, 2000], [8, 14, 2021], [9, 21, 2024], [11, 27, 2026], [3, 30, 2021], [7, 21, 2014]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This function allows for modifying the date  of a booking entry.  This allows for us to change from one booking entry date to another.  This allow allow for the us to continue booking entires as required.  </t>
+  </si>
+  <si>
+    <t>The parameters include the name of the person who were are moving the booking entry for.  The other is the original room.  The next is the original date.  Then the next is the new date and time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function outputs true if the function works as intended.  The function outputs false if the program fails to work as intended.  This means they they are giving a true or false for the given options in the function.  </t>
+  </si>
+  <si>
+    <t>Float, Float, Float, Float, Float, Float, Float, Float, Float, Float</t>
+  </si>
+  <si>
+    <t>202031, 212341, 202453, 212658, 212891, 234567, 233212, 232345, 256781, 256781</t>
+  </si>
+  <si>
+    <t>Sally, Bern, Keith, Harvey, Sam, Drake, Eithan, Lee, Nick, Jack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This function allows for scheduling a booking entry.  It does so by changing the booking play to work as intended.  It can also assign a ID to the booking entry so the booking entry will be change as required.  This make sure the task works as intended.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The outputs for the function are true when the function is able to schedule the task successful.  The function booking entry is false when the booking entry is not able to schedule the task as intended.  This allows for us to test if the function is working as intended.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resevered space for legacy code.  Not required and will not be used in testing the code in of this program.  Backwards compability with the rest of the project.  </t>
+  </si>
+  <si>
+    <t>String, String, String, String, String, String, String, String</t>
+  </si>
+  <si>
+    <t>"Saving user data.", "Saving user password.", "Saving users name.", "Saving user values", "Saving user location.", "Saving user history.", "Saving user birthdate.", "Saving user goverement id information.", "Saving users finicial record.", "Saving users task history."</t>
+  </si>
+  <si>
+    <t>Bool, Bool, Bool, Bool, Bool, Bool, Bool, Bool, Bool, Bool, Bool</t>
+  </si>
+  <si>
+    <t>True, False, True, True, False, False, True, True, True,  True, False</t>
+  </si>
+  <si>
+    <t>True, True, True, True, True, True, True, True, True, True, True</t>
+  </si>
+  <si>
+    <t>The data saving policy allows for you to change which data is saved by the program.  You choices for saving data effect the state of the program you are using.  It changes what data the organization can save and alter.  This changes the program and shifts the way it works overall as a direct result.</t>
+  </si>
+  <si>
+    <t>The parameters of the function include the booking ID, the room number, the date of the booking entry, and, the name of the users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The parameters for the function are the first parameter which is the name of the data saving policy.  The second parameters is the state of the data saving policy.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function output returns true when the function has returned the correct information.  It returns false when the function has failed to return the correct information.  This makes sure the program works as intended.  </t>
+  </si>
+  <si>
+    <t>"Saving user data.", "Saving user password.", "Saving users name.", "Saving user values", "Saving user location.", "Saving user history.", "Saving user birthdate.", "Saving user goverement id information.", "Saving users finicial record.", "Saving users t</t>
+  </si>
+  <si>
+    <t>False, True, False, False, True, False, True, True, False, False, False</t>
+  </si>
+  <si>
+    <t>The process of mutated the data saving policy.  This change the data saving policy to make sure it works as intended.  By altering the data saving policy we can ensure that the program is working as intended.  This will also give users the chance to alter the what the program is saving and which data bases processes it sees.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The parameters for the function are the name of the data saving policy and the state the users would like to no be set to.  The first parameter test if the data saving policies is correctly selected.  The second select if the correct users data is being saved.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function outputs true when the update has been successful.  The function updates false when the function has been unsucessful.  This allows for use to make sure to understand the differences between successful and unsucessful updates.   </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -761,6 +890,12 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -787,9 +922,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1707,7 +1843,7 @@
       </c>
     </row>
     <row r="7" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>97</v>
       </c>
       <c r="C7" t="s">
@@ -1733,7 +1869,7 @@
       </c>
     </row>
     <row r="8" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C8" t="s">
@@ -1742,9 +1878,30 @@
       <c r="E8">
         <v>1</v>
       </c>
+      <c r="H8" t="s">
+        <v>86</v>
+      </c>
+      <c r="J8" t="s">
+        <v>235</v>
+      </c>
+      <c r="BF8" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI8" t="s">
+        <v>214</v>
+      </c>
+      <c r="BL8" t="s">
+        <v>236</v>
+      </c>
+      <c r="BO8" t="s">
+        <v>237</v>
+      </c>
+      <c r="BR8" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="9" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>101</v>
       </c>
       <c r="C9" t="s">
@@ -1753,82 +1910,307 @@
       <c r="E9">
         <v>1</v>
       </c>
+      <c r="H9" t="s">
+        <v>86</v>
+      </c>
+      <c r="J9" t="s">
+        <v>235</v>
+      </c>
+      <c r="BF9" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI9" t="s">
+        <v>214</v>
+      </c>
+      <c r="BL9" t="s">
+        <v>239</v>
+      </c>
+      <c r="BO9" t="s">
+        <v>240</v>
+      </c>
+      <c r="BR9" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="10" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>103</v>
       </c>
       <c r="C10" t="s">
         <v>104</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="H10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J10" t="s">
+        <v>242</v>
+      </c>
+      <c r="M10" t="s">
+        <v>243</v>
+      </c>
+      <c r="O10" t="s">
+        <v>244</v>
+      </c>
+      <c r="R10" t="s">
+        <v>245</v>
+      </c>
+      <c r="T10" t="s">
+        <v>246</v>
+      </c>
+      <c r="BF10" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI10" t="s">
+        <v>214</v>
+      </c>
+      <c r="BL10" t="s">
+        <v>247</v>
+      </c>
+      <c r="BO10" t="s">
+        <v>248</v>
+      </c>
+      <c r="BR10" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="11" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>105</v>
       </c>
       <c r="C11" t="s">
         <v>106</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="H11" t="s">
+        <v>86</v>
+      </c>
+      <c r="J11" t="s">
+        <v>242</v>
+      </c>
+      <c r="M11" t="s">
+        <v>243</v>
+      </c>
+      <c r="O11" t="s">
+        <v>244</v>
+      </c>
+      <c r="R11" t="s">
+        <v>245</v>
+      </c>
+      <c r="T11" t="s">
+        <v>246</v>
+      </c>
+      <c r="BF11" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI11" t="s">
+        <v>214</v>
+      </c>
+      <c r="BL11" t="s">
+        <v>250</v>
+      </c>
+      <c r="BO11" t="s">
+        <v>251</v>
+      </c>
+      <c r="BR11" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="12" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C12" t="s">
         <v>108</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="H12" t="s">
+        <v>86</v>
+      </c>
+      <c r="J12" t="s">
+        <v>242</v>
+      </c>
+      <c r="M12" t="s">
+        <v>243</v>
+      </c>
+      <c r="O12" t="s">
+        <v>244</v>
+      </c>
+      <c r="R12" t="s">
+        <v>245</v>
+      </c>
+      <c r="T12" t="s">
+        <v>246</v>
+      </c>
+      <c r="W12" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>254</v>
+      </c>
+      <c r="BF12" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI12" t="s">
+        <v>214</v>
+      </c>
+      <c r="BL12" t="s">
+        <v>255</v>
+      </c>
+      <c r="BO12" t="s">
+        <v>256</v>
+      </c>
+      <c r="BR12" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>109</v>
       </c>
       <c r="C13" t="s">
         <v>110</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="H13" t="s">
+        <v>258</v>
+      </c>
+      <c r="J13" t="s">
+        <v>259</v>
+      </c>
+      <c r="M13" t="s">
+        <v>243</v>
+      </c>
+      <c r="O13" t="s">
+        <v>244</v>
+      </c>
+      <c r="R13" t="s">
+        <v>245</v>
+      </c>
+      <c r="T13" t="s">
+        <v>246</v>
+      </c>
+      <c r="W13" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>260</v>
+      </c>
+      <c r="BF13" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI13" t="s">
+        <v>214</v>
+      </c>
+      <c r="BL13" t="s">
+        <v>261</v>
+      </c>
+      <c r="BO13" t="s">
+        <v>270</v>
+      </c>
+      <c r="BR13" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="14" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C14" t="s">
+      <c r="B14" s="1"/>
+      <c r="C14" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E14">
-        <v>4</v>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="BL14" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="15" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>113</v>
       </c>
+      <c r="B15" s="1"/>
       <c r="C15" t="s">
         <v>114</v>
       </c>
-      <c r="E15">
-        <v>1</v>
+      <c r="E15" s="2">
+        <v>2</v>
+      </c>
+      <c r="H15" t="s">
+        <v>264</v>
+      </c>
+      <c r="J15" t="s">
+        <v>265</v>
+      </c>
+      <c r="M15" t="s">
+        <v>266</v>
+      </c>
+      <c r="O15" t="s">
+        <v>267</v>
+      </c>
+      <c r="BF15" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI15" t="s">
+        <v>268</v>
+      </c>
+      <c r="BL15" t="s">
+        <v>269</v>
+      </c>
+      <c r="BO15" t="s">
+        <v>271</v>
+      </c>
+      <c r="BR15" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="16" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>115</v>
       </c>
       <c r="C16" t="s">
         <v>116</v>
       </c>
-      <c r="E16">
-        <v>1</v>
+      <c r="E16" s="2">
+        <v>2</v>
+      </c>
+      <c r="H16" t="s">
+        <v>264</v>
+      </c>
+      <c r="J16" t="s">
+        <v>273</v>
+      </c>
+      <c r="M16" t="s">
+        <v>266</v>
+      </c>
+      <c r="O16" t="s">
+        <v>274</v>
+      </c>
+      <c r="BF16" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI16" t="s">
+        <v>268</v>
+      </c>
+      <c r="BL16" t="s">
+        <v>275</v>
+      </c>
+      <c r="BO16" t="s">
+        <v>276</v>
+      </c>
+      <c r="BR16" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added Update: Added updated function.
I added updated function to the system.  I am not make sure the program works as intended.
</commit_message>
<xml_diff>
--- a/Test-Cases/Testing-Script-Records.xlsx
+++ b/Test-Cases/Testing-Script-Records.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11023"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexahope/Documents/GitHub/Ophelias-Oasis/Test-Cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE61DDA-9E21-4B45-8BDA-E4D5599A02D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B0C1C7-B2D3-2144-91C4-00AF8BF9BEA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" firstSheet="1" activeTab="1" xr2:uid="{32C5AFC3-1601-AE47-BE56-3877807D3FAA}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="311">
   <si>
     <t>Transaction ID:</t>
   </si>
@@ -874,13 +874,112 @@
   </si>
   <si>
     <t xml:space="preserve">The function outputs true when the update has been successful.  The function updates false when the function has been unsucessful.  This allows for use to make sure to understand the differences between successful and unsucessful updates.   </t>
+  </si>
+  <si>
+    <t>"Speech to Text", "Speech to Text", "Dark Mode", "Light Mode", "Voiceover Mode", "Offline Mode", "Stick Keys Mode", "Inverted Color Mode", "Speech to Text", "Text to Speech"</t>
+  </si>
+  <si>
+    <t>The process of mutated which accomdation are being used at any given point in time.  This alters what the system is doing so everyone can be happy using it.  This system test if the accomdation are being accurately tested.  This allows for the interface to be test as much as possible.</t>
+  </si>
+  <si>
+    <t>The parameters for the function are the name of the accomdation.  This parameter allows for editing the accomdation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The output is a binary value which is true if the system has changed it and false if the system has failed.  </t>
+  </si>
+  <si>
+    <t>The process of disabililing accomdation.  This process allows for us to understand if the accomdation are working as intended.  This way we can work out the accomdatio if required.  I am making sure that every bit of the program can be activated and deactivate.</t>
+  </si>
+  <si>
+    <t>The parameter allows for editing the accomdation setting.  The accomdation allows for the system to test if the accomdation are being edited correct.  This way we can see if the accomdation are being activated and deactivated as intended.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The output is a binary output which is true when the function has disabiled the accomdation.  It is false when the system has failed to do this action.  </t>
+  </si>
+  <si>
+    <t>"Track1p1.mp3", "Track1p2.mp3", "Track2s1.mp3", "Track2s2.mp3", "Track3s1.mp3", "Track3s2.mp3", "Track4s1.mp3", "Track4s2.mp3", "Track5s1.mp3", "Track5s2.mp3"</t>
+  </si>
+  <si>
+    <t>"A great brown bear jumps over a pink fox.", "A great brown bear jumps over a pink fox.", "A brown duck crosses the river.", "A brown duck crosses the river.", "A fox jumps over the hen house across the country.  The country is old and dark and grey.  The fox has a hard time seeing.  This is the impact of the woods.", "A fox jumps over the hen house across the country.  The country is old and dark and grey.  The fox has a hard time seeing.  This is the impact of the woods.", "A steel wool jacked make the best food.", "A steel wool jacked make the best food.", "A good night for trick-or-treating.  But who is ringing on your doorbell?", "A good night for trick-or-treating.  But who is ringing on your doorbell?"</t>
+  </si>
+  <si>
+    <t>This function is for taking speech files from the system.  It analysis them and them preforms speech to text conversion. It then records if the convversion has been successful.</t>
+  </si>
+  <si>
+    <t>The parameter is for determine where the location of the speech file is.  Once we locate it we can edit it to make sure the file contains the correct data.  It can then open the speech to text file and then analysis it and return the text from inside the file.</t>
+  </si>
+  <si>
+    <t>The output for the function is the text conversion of the text in the file.  It is used for understand if the file contains the correct content and analysis it to make sure the correct amount of data is stored in the file.</t>
+  </si>
+  <si>
+    <t>This function converts text to speech files.  It then outputs a file that should look like the file from before.  This software looks over the file and determine if the function is returning true as it should. Then it make sure the program is functioning as intended.</t>
+  </si>
+  <si>
+    <t>The parameter for the function is the string containing the different string we would like to convert from speech to text.  The files are stored locally.  Then the system determine if it has worded as intended using the funciton and returns true if it has a false if it has not.</t>
+  </si>
+  <si>
+    <t>The output is true if the function has create a music file contain the correct speech.  The file is false if it cannot do so due to issues in the program.</t>
+  </si>
+  <si>
+    <t>"Sally@EmuSoftware.com", "Bern@EmuSoftware.com", "Keith@EmuSoftware.com", "Harvey@EmuSoftware.com", "Sam@EmuSoftware.com", "Drake@EmuSoftware.com", "Eithan@EmuSoftware.com", "Lee@EmuSoftware.com", "Nick@EmuSoftware.com", "Jack@EmuSoftware.com"</t>
+  </si>
+  <si>
+    <t>This function is used to send a confirmation report about users.  It is used to determine if the user receives the confirmation report or not.</t>
+  </si>
+  <si>
+    <t>The parameter for the function is the email.  This isused do determine who to send the python confirmation report to.</t>
+  </si>
+  <si>
+    <t>The output for the function is true if the confirmation report sends as required.  It is false if the confirmation report does not send as intended.</t>
+  </si>
+  <si>
+    <t>True, False, True, False, True, False, True, False, True, False</t>
+  </si>
+  <si>
+    <t>This function determine if the confirmation report has been received.  If it has it return true.  If it has not it does not return anything.</t>
+  </si>
+  <si>
+    <t>There are no parameter since we are not receiving it form one person.</t>
+  </si>
+  <si>
+    <t>The output for the function is a boolean value which is true when the confirmation report is received.  It is false when it has not been received.</t>
+  </si>
+  <si>
+    <t>"Sally@EmuSoftware.com", "Bern@EmuSoftware.com", "Keith@EmuSoftware.com", "Harvey@EmuSoftware.com", "Sam@EmuSoftware.com", "Drake@EmuSoftware.com", "Eithan@EmuSoftware.com", "Lee@EmuSoftware.com", Nick@EmuSoftware.com", "Jack@EmuSoftware.com"</t>
+  </si>
+  <si>
+    <t>"Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed."</t>
+  </si>
+  <si>
+    <t>This function allows for the encoding of the confirmation report into a string.  It then make sure to return the string to the user.  If everything goes according to play the user will be able to see the message.  It means that the system will generate a small profit for it use.</t>
+  </si>
+  <si>
+    <t>There is one parameter which say the name of the user who confirmation message to report.  By doing this it will allow for us to determine if the right users confirmation page is being report.  This will allow for the correct message to be selected.  The latest confirmation message for that user should be returned in the testing cases.</t>
+  </si>
+  <si>
+    <t>The output is the lastest confirmation message for the user.  This should be return due to the system requesting it.</t>
+  </si>
+  <si>
+    <t>[9, 27, 26], [9, 27, 26], [9, 27, 26], [9, 27, 26], [9, 27, 26], [9, 27, 26], [9, 27, 26], [9, 27, 26], [9, 27, 26], [9, 27, 26]</t>
+  </si>
+  <si>
+    <t>Confirmation Report: We are pleased to receive you message and you order has been confirmed., "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed.", "Confirmation Report: We are pleased to receive you message and you order has been confirmed."</t>
+  </si>
+  <si>
+    <t>The function will return the current date on the confirmation message.  If the message matches the system date the the system will do fine.  We should see the same message on the system.  However, the message can change based on what is occuring in the system.</t>
+  </si>
+  <si>
+    <t>The is one parameter that contains the message for the user.  It should what is currently happening from the perspective of the user.</t>
+  </si>
+  <si>
+    <t>The output for the function is the latest date.  It should what the latest date on the message was.  This will allow for the system to understand when the message was sent and if it was sent on the same day.  If it was a later version of the program will say it has been successful at passing this test.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -898,6 +997,28 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -919,15 +1040,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2213,8 +2339,8 @@
         <v>277</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="17" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
         <v>117</v>
       </c>
       <c r="C17" t="s">
@@ -2223,9 +2349,30 @@
       <c r="E17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="H17" t="s">
+        <v>264</v>
+      </c>
+      <c r="J17" t="s">
+        <v>278</v>
+      </c>
+      <c r="BF17" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI17" t="s">
+        <v>268</v>
+      </c>
+      <c r="BL17" t="s">
+        <v>279</v>
+      </c>
+      <c r="BO17" t="s">
+        <v>280</v>
+      </c>
+      <c r="BR17" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="18" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>119</v>
       </c>
       <c r="C18" t="s">
@@ -2234,9 +2381,30 @@
       <c r="E18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="H18" t="s">
+        <v>264</v>
+      </c>
+      <c r="J18" t="s">
+        <v>278</v>
+      </c>
+      <c r="BF18" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI18" t="s">
+        <v>268</v>
+      </c>
+      <c r="BL18" t="s">
+        <v>282</v>
+      </c>
+      <c r="BO18" t="s">
+        <v>283</v>
+      </c>
+      <c r="BR18" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="19" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>121</v>
       </c>
       <c r="C19" t="s">
@@ -2245,9 +2413,30 @@
       <c r="E19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="H19" t="s">
+        <v>264</v>
+      </c>
+      <c r="J19" t="s">
+        <v>285</v>
+      </c>
+      <c r="BF19" t="s">
+        <v>86</v>
+      </c>
+      <c r="BI19" t="s">
+        <v>286</v>
+      </c>
+      <c r="BL19" t="s">
+        <v>287</v>
+      </c>
+      <c r="BO19" t="s">
+        <v>288</v>
+      </c>
+      <c r="BR19" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="20" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>123</v>
       </c>
       <c r="C20" t="s">
@@ -2256,9 +2445,30 @@
       <c r="E20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="H20" t="s">
+        <v>264</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="BF20" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI20" t="s">
+        <v>268</v>
+      </c>
+      <c r="BL20" t="s">
+        <v>290</v>
+      </c>
+      <c r="BO20" t="s">
+        <v>291</v>
+      </c>
+      <c r="BR20" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="21" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>125</v>
       </c>
       <c r="C21" t="s">
@@ -2267,20 +2477,56 @@
       <c r="E21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="H21" t="s">
+        <v>264</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="BF21" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI21" t="s">
+        <v>268</v>
+      </c>
+      <c r="BL21" t="s">
+        <v>294</v>
+      </c>
+      <c r="BO21" t="s">
+        <v>295</v>
+      </c>
+      <c r="BR21" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="22" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>127</v>
       </c>
       <c r="C22" t="s">
         <v>128</v>
       </c>
       <c r="E22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+      <c r="BF22" t="s">
+        <v>213</v>
+      </c>
+      <c r="BI22" t="s">
+        <v>297</v>
+      </c>
+      <c r="BL22" t="s">
+        <v>298</v>
+      </c>
+      <c r="BO22" t="s">
+        <v>299</v>
+      </c>
+      <c r="BR22" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="23" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
         <v>129</v>
       </c>
       <c r="C23" t="s">
@@ -2289,9 +2535,30 @@
       <c r="E23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="H23" t="s">
+        <v>86</v>
+      </c>
+      <c r="J23" t="s">
+        <v>301</v>
+      </c>
+      <c r="BF23" t="s">
+        <v>86</v>
+      </c>
+      <c r="BI23" t="s">
+        <v>302</v>
+      </c>
+      <c r="BL23" t="s">
+        <v>303</v>
+      </c>
+      <c r="BO23" t="s">
+        <v>304</v>
+      </c>
+      <c r="BR23" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="24" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
         <v>131</v>
       </c>
       <c r="C24" t="s">
@@ -2300,8 +2567,29 @@
       <c r="E24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H24" t="s">
+        <v>86</v>
+      </c>
+      <c r="J24" t="s">
+        <v>307</v>
+      </c>
+      <c r="BF24" t="s">
+        <v>245</v>
+      </c>
+      <c r="BI24" t="s">
+        <v>306</v>
+      </c>
+      <c r="BL24" t="s">
+        <v>308</v>
+      </c>
+      <c r="BO24" t="s">
+        <v>309</v>
+      </c>
+      <c r="BR24" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="25" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>133</v>
       </c>
@@ -2312,7 +2600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>135</v>
       </c>
@@ -2323,7 +2611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>137</v>
       </c>
@@ -2334,7 +2622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>139</v>
       </c>
@@ -2345,7 +2633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>141</v>
       </c>
@@ -2356,7 +2644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>143</v>
       </c>
@@ -2367,7 +2655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>145</v>
       </c>
@@ -2378,7 +2666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>147</v>
       </c>
@@ -2720,6 +3008,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J21" r:id="rId1" display="Sally@EmuSoftware.Com" xr:uid="{89E1025F-7416-854B-BFAE-C980E993CAED}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: Current version of program.
Update the current program to the currently working version.  I will not update the debugger as well.
</commit_message>
<xml_diff>
--- a/Test-Cases/Testing-Script-Records.xlsx
+++ b/Test-Cases/Testing-Script-Records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexahope/Documents/GitHub/Ophelias-Oasis/Test-Cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0AEEC07-C1E8-8A43-9801-B8B23410461F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8457345-59F6-F145-9DA9-1EB50F273981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" firstSheet="1" activeTab="1" xr2:uid="{32C5AFC3-1601-AE47-BE56-3877807D3FAA}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="272">
   <si>
     <t>Transaction ID:</t>
   </si>
@@ -324,9 +324,6 @@
     <t xml:space="preserve">Function 4:  </t>
   </si>
   <si>
-    <t>displayMenuAdviseHelpMenu</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 5:  </t>
   </si>
   <si>
@@ -396,27 +393,15 @@
     <t xml:space="preserve">Function 16:  </t>
   </si>
   <si>
-    <t>enableAccomdation</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 17:  </t>
   </si>
   <si>
-    <t>deleteAccomdation</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 18:  </t>
   </si>
   <si>
-    <t>speechToText</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 19:  </t>
   </si>
   <si>
-    <t>textToSpeech</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 20:  </t>
   </si>
   <si>
@@ -468,27 +453,15 @@
     <t xml:space="preserve">Function 28:  </t>
   </si>
   <si>
-    <t>modifyLogo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 29:  </t>
   </si>
   <si>
-    <t>hideLogo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 30:  </t>
   </si>
   <si>
-    <t>showLogo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 31:  </t>
   </si>
   <si>
-    <t>reserve</t>
-  </si>
-  <si>
     <t xml:space="preserve">Function 32:  </t>
   </si>
   <si>
@@ -528,144 +501,33 @@
     <t xml:space="preserve">Function 38:  </t>
   </si>
   <si>
-    <t>trackSupply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 39:  </t>
-  </si>
-  <si>
-    <t>deleteSupply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 40:  </t>
-  </si>
-  <si>
-    <t>changeSupply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 41:  </t>
-  </si>
-  <si>
-    <t>addSupply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 42:  </t>
-  </si>
-  <si>
     <t>transaction</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 43:  </t>
-  </si>
-  <si>
     <t>addNewTransaction</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 44:  </t>
-  </si>
-  <si>
     <t>deleteTransaction</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 45:  </t>
-  </si>
-  <si>
     <t>modifyTransaction</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 46:  </t>
-  </si>
-  <si>
-    <t>readUserProfile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 47:  </t>
-  </si>
-  <si>
-    <t>writeUserProfile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 48:  </t>
-  </si>
-  <si>
     <t>modifyUserProfile</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 49:  </t>
-  </si>
-  <si>
     <t>deleteUserProfile</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 50:  </t>
-  </si>
-  <si>
     <t>displayConfirmationCode</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 51:  </t>
-  </si>
-  <si>
     <t>minimizeQRCode</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 52:  </t>
-  </si>
-  <si>
-    <t>recordRetaiment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 53:  </t>
-  </si>
-  <si>
-    <t>modifyRetainment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 54:  </t>
-  </si>
-  <si>
-    <t>deleteRetainment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 55:  </t>
-  </si>
-  <si>
-    <t>viewRetainment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 56:  </t>
-  </si>
-  <si>
-    <t>changeReportedReservation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 59:  </t>
-  </si>
-  <si>
-    <t>deleteReportedReservation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 60:  </t>
-  </si>
-  <si>
-    <t>reportReservationPrice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 61:  </t>
-  </si>
-  <si>
-    <t>changePriceReservation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Function 62:  </t>
-  </si>
-  <si>
     <t>deletePriceReservation</t>
   </si>
   <si>
-    <t xml:space="preserve">Function 63:  </t>
-  </si>
-  <si>
     <t>addReportedReservationPricing</t>
   </si>
   <si>
@@ -717,15 +579,6 @@
     <t xml:space="preserve">The output is a string returning the complete history of the person.  This will allow for the user to understand how their accomdation and needs changes over time.  </t>
   </si>
   <si>
-    <t>"printReport: Display a report of a given fuction.", "changeAccBillReports: The function testes the ability for the program to change the accomdation billing report.", "returnHistOfAccReport: The software ability to report on backups in the program of the different users.", "displayMenuAdviseHelpMenu: This function is used to display help menu and options for the different functions.", "createBackup: The function to create a backup of the local operating parameters.", "displayHelpMenu: A function for displaying the help menu for the current program.", "storeBackup: The function for storing a backup of the local system configuration.", "deleteBackup: The function for deleting the backup of the software function as intended.", "createBookingEntry: A function for creating booking entry in the larger system.", "deleteBookingEntry: A function for deleting booking entries on the local system."</t>
-  </si>
-  <si>
-    <t>The function is used for printing a local help menu so that we can understand if the function is working as it is intended to work.  It will allow for the function to be programmed as intended and work as it was intended to work.</t>
-  </si>
-  <si>
-    <t>The output of the function for each case is the help menu.  The program displays the help menu during this process and make sure the help menu works as it is intended to work.</t>
-  </si>
-  <si>
     <t>The function is called to create a local backup of the whole program.  This make sure the program works as intended and allow for a local backup of the whole program as a direct result.</t>
   </si>
   <si>
@@ -876,51 +729,6 @@
     <t xml:space="preserve">The function outputs true when the update has been successful.  The function updates false when the function has been unsucessful.  This allows for use to make sure to understand the differences between successful and unsucessful updates.   </t>
   </si>
   <si>
-    <t>"Speech to Text", "Speech to Text", "Dark Mode", "Light Mode", "Voiceover Mode", "Offline Mode", "Stick Keys Mode", "Inverted Color Mode", "Speech to Text", "Text to Speech"</t>
-  </si>
-  <si>
-    <t>The process of mutated which accomdation are being used at any given point in time.  This alters what the system is doing so everyone can be happy using it.  This system test if the accomdation are being accurately tested.  This allows for the interface to be test as much as possible.</t>
-  </si>
-  <si>
-    <t>The parameters for the function are the name of the accomdation.  This parameter allows for editing the accomdation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The output is a binary value which is true if the system has changed it and false if the system has failed.  </t>
-  </si>
-  <si>
-    <t>The process of disabililing accomdation.  This process allows for us to understand if the accomdation are working as intended.  This way we can work out the accomdatio if required.  I am making sure that every bit of the program can be activated and deactivate.</t>
-  </si>
-  <si>
-    <t>The parameter allows for editing the accomdation setting.  The accomdation allows for the system to test if the accomdation are being edited correct.  This way we can see if the accomdation are being activated and deactivated as intended.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The output is a binary output which is true when the function has disabiled the accomdation.  It is false when the system has failed to do this action.  </t>
-  </si>
-  <si>
-    <t>"Track1p1.mp3", "Track1p2.mp3", "Track2s1.mp3", "Track2s2.mp3", "Track3s1.mp3", "Track3s2.mp3", "Track4s1.mp3", "Track4s2.mp3", "Track5s1.mp3", "Track5s2.mp3"</t>
-  </si>
-  <si>
-    <t>"A great brown bear jumps over a pink fox.", "A great brown bear jumps over a pink fox.", "A brown duck crosses the river.", "A brown duck crosses the river.", "A fox jumps over the hen house across the country.  The country is old and dark and grey.  The fox has a hard time seeing.  This is the impact of the woods.", "A fox jumps over the hen house across the country.  The country is old and dark and grey.  The fox has a hard time seeing.  This is the impact of the woods.", "A steel wool jacked make the best food.", "A steel wool jacked make the best food.", "A good night for trick-or-treating.  But who is ringing on your doorbell?", "A good night for trick-or-treating.  But who is ringing on your doorbell?"</t>
-  </si>
-  <si>
-    <t>This function is for taking speech files from the system.  It analysis them and them preforms speech to text conversion. It then records if the convversion has been successful.</t>
-  </si>
-  <si>
-    <t>The parameter is for determine where the location of the speech file is.  Once we locate it we can edit it to make sure the file contains the correct data.  It can then open the speech to text file and then analysis it and return the text from inside the file.</t>
-  </si>
-  <si>
-    <t>The output for the function is the text conversion of the text in the file.  It is used for understand if the file contains the correct content and analysis it to make sure the correct amount of data is stored in the file.</t>
-  </si>
-  <si>
-    <t>This function converts text to speech files.  It then outputs a file that should look like the file from before.  This software looks over the file and determine if the function is returning true as it should. Then it make sure the program is functioning as intended.</t>
-  </si>
-  <si>
-    <t>The parameter for the function is the string containing the different string we would like to convert from speech to text.  The files are stored locally.  Then the system determine if it has worded as intended using the funciton and returns true if it has a false if it has not.</t>
-  </si>
-  <si>
-    <t>The output is true if the function has create a music file contain the correct speech.  The file is false if it cannot do so due to issues in the program.</t>
-  </si>
-  <si>
     <t>"Sally@EmuSoftware.com", "Bern@EmuSoftware.com", "Keith@EmuSoftware.com", "Harvey@EmuSoftware.com", "Sam@EmuSoftware.com", "Drake@EmuSoftware.com", "Eithan@EmuSoftware.com", "Lee@EmuSoftware.com", "Nick@EmuSoftware.com", "Jack@EmuSoftware.com"</t>
   </si>
   <si>
@@ -975,18 +783,6 @@
     <t>The output for the function is the latest date.  It should what the latest date on the message was.  This will allow for the system to understand when the message was sent and if it was sent on the same day.  If it was a later version of the program will say it has been successful at passing this test.</t>
   </si>
   <si>
-    <t>Function 64:</t>
-  </si>
-  <si>
-    <t>Function 65:</t>
-  </si>
-  <si>
-    <t>Function 66:</t>
-  </si>
-  <si>
-    <t>Function 67:</t>
-  </si>
-  <si>
     <t>getDaysInAdvance</t>
   </si>
   <si>
@@ -1048,13 +844,25 @@
   </si>
   <si>
     <t>The are not paremeter for the function.  We are just using the data being returned.</t>
+  </si>
+  <si>
+    <t>Function 39:</t>
+  </si>
+  <si>
+    <t>Function 40:</t>
+  </si>
+  <si>
+    <t>Function 41:</t>
+  </si>
+  <si>
+    <t>Function 42:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1079,13 +887,6 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1119,13 +920,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1780,7 +1580,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44E41573-350E-4D19-A26B-D0AE87797D6F}">
-  <dimension ref="A1:BR66"/>
+  <dimension ref="A1:BR43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="20.6640625" customWidth="1"/>
@@ -1894,13 +1694,13 @@
         <v>88</v>
       </c>
       <c r="BL2" t="s">
-        <v>215</v>
+        <v>169</v>
       </c>
       <c r="BO2" t="s">
-        <v>216</v>
+        <v>170</v>
       </c>
       <c r="BR2" t="s">
-        <v>217</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:70" x14ac:dyDescent="0.2">
@@ -1917,34 +1717,34 @@
         <v>86</v>
       </c>
       <c r="J3" t="s">
-        <v>209</v>
+        <v>163</v>
       </c>
       <c r="M3" t="s">
-        <v>210</v>
+        <v>164</v>
       </c>
       <c r="O3" t="s">
-        <v>211</v>
+        <v>165</v>
       </c>
       <c r="R3" t="s">
         <v>86</v>
       </c>
       <c r="T3" t="s">
-        <v>212</v>
+        <v>166</v>
       </c>
       <c r="BF3" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI3" t="s">
-        <v>214</v>
+        <v>168</v>
       </c>
       <c r="BL3" t="s">
-        <v>218</v>
+        <v>172</v>
       </c>
       <c r="BO3" t="s">
-        <v>219</v>
+        <v>173</v>
       </c>
       <c r="BR3" t="s">
-        <v>220</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:70" x14ac:dyDescent="0.2">
@@ -1961,22 +1761,22 @@
         <v>86</v>
       </c>
       <c r="J4" t="s">
-        <v>209</v>
+        <v>163</v>
       </c>
       <c r="BF4" t="s">
         <v>86</v>
       </c>
       <c r="BI4" t="s">
-        <v>221</v>
+        <v>175</v>
       </c>
       <c r="BL4" t="s">
-        <v>222</v>
+        <v>176</v>
       </c>
       <c r="BO4" t="s">
-        <v>223</v>
+        <v>177</v>
       </c>
       <c r="BR4" t="s">
-        <v>224</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:70" x14ac:dyDescent="0.2">
@@ -1984,7 +1784,7 @@
         <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -1993,88 +1793,88 @@
         <v>86</v>
       </c>
       <c r="J5" t="s">
-        <v>87</v>
+        <v>163</v>
       </c>
       <c r="BF5" t="s">
-        <v>86</v>
+        <v>167</v>
       </c>
       <c r="BI5" t="s">
-        <v>225</v>
+        <v>168</v>
       </c>
       <c r="BL5" t="s">
-        <v>226</v>
+        <v>179</v>
       </c>
       <c r="BO5" t="s">
-        <v>216</v>
+        <v>180</v>
       </c>
       <c r="BR5" t="s">
-        <v>227</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="H6" t="s">
+        <v>0</v>
+      </c>
+      <c r="BF6" t="s">
         <v>86</v>
       </c>
-      <c r="J6" t="s">
-        <v>209</v>
-      </c>
-      <c r="BF6" t="s">
-        <v>213</v>
-      </c>
       <c r="BI6" t="s">
-        <v>214</v>
+        <v>182</v>
       </c>
       <c r="BL6" t="s">
-        <v>228</v>
+        <v>183</v>
       </c>
       <c r="BO6" t="s">
-        <v>229</v>
+        <v>184</v>
       </c>
       <c r="BR6" t="s">
-        <v>230</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>86</v>
+      </c>
+      <c r="J7" t="s">
+        <v>186</v>
       </c>
       <c r="BF7" t="s">
-        <v>86</v>
+        <v>167</v>
       </c>
       <c r="BI7" t="s">
-        <v>231</v>
+        <v>168</v>
       </c>
       <c r="BL7" t="s">
-        <v>232</v>
+        <v>187</v>
       </c>
       <c r="BO7" t="s">
-        <v>233</v>
+        <v>188</v>
       </c>
       <c r="BR7" t="s">
-        <v>234</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2083,62 +1883,74 @@
         <v>86</v>
       </c>
       <c r="J8" t="s">
-        <v>235</v>
+        <v>186</v>
       </c>
       <c r="BF8" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI8" t="s">
-        <v>214</v>
+        <v>168</v>
       </c>
       <c r="BL8" t="s">
-        <v>236</v>
+        <v>190</v>
       </c>
       <c r="BO8" t="s">
-        <v>237</v>
+        <v>191</v>
       </c>
       <c r="BR8" t="s">
-        <v>238</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H9" t="s">
         <v>86</v>
       </c>
       <c r="J9" t="s">
-        <v>235</v>
+        <v>193</v>
+      </c>
+      <c r="M9" t="s">
+        <v>194</v>
+      </c>
+      <c r="O9" t="s">
+        <v>195</v>
+      </c>
+      <c r="R9" t="s">
+        <v>196</v>
+      </c>
+      <c r="T9" t="s">
+        <v>197</v>
       </c>
       <c r="BF9" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI9" t="s">
-        <v>214</v>
+        <v>168</v>
       </c>
       <c r="BL9" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
       <c r="BO9" t="s">
-        <v>240</v>
+        <v>199</v>
       </c>
       <c r="BR9" t="s">
-        <v>241</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -2147,529 +1959,412 @@
         <v>86</v>
       </c>
       <c r="J10" t="s">
-        <v>242</v>
+        <v>193</v>
       </c>
       <c r="M10" t="s">
-        <v>243</v>
+        <v>194</v>
       </c>
       <c r="O10" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="R10" t="s">
-        <v>245</v>
+        <v>196</v>
       </c>
       <c r="T10" t="s">
-        <v>246</v>
+        <v>197</v>
       </c>
       <c r="BF10" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI10" t="s">
-        <v>214</v>
+        <v>168</v>
       </c>
       <c r="BL10" t="s">
-        <v>247</v>
+        <v>201</v>
       </c>
       <c r="BO10" t="s">
-        <v>248</v>
+        <v>202</v>
       </c>
       <c r="BR10" t="s">
-        <v>249</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H11" t="s">
         <v>86</v>
       </c>
       <c r="J11" t="s">
-        <v>242</v>
+        <v>193</v>
       </c>
       <c r="M11" t="s">
-        <v>243</v>
+        <v>194</v>
       </c>
       <c r="O11" t="s">
-        <v>244</v>
+        <v>195</v>
       </c>
       <c r="R11" t="s">
-        <v>245</v>
+        <v>196</v>
       </c>
       <c r="T11" t="s">
-        <v>246</v>
+        <v>197</v>
+      </c>
+      <c r="W11" t="s">
+        <v>204</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>205</v>
       </c>
       <c r="BF11" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI11" t="s">
-        <v>214</v>
+        <v>168</v>
       </c>
       <c r="BL11" t="s">
-        <v>250</v>
+        <v>206</v>
       </c>
       <c r="BO11" t="s">
-        <v>251</v>
+        <v>207</v>
       </c>
       <c r="BR11" t="s">
-        <v>252</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H12" t="s">
+        <v>209</v>
+      </c>
+      <c r="J12" t="s">
+        <v>210</v>
+      </c>
+      <c r="M12" t="s">
+        <v>194</v>
+      </c>
+      <c r="O12" t="s">
+        <v>195</v>
+      </c>
+      <c r="R12" t="s">
+        <v>196</v>
+      </c>
+      <c r="T12" t="s">
+        <v>197</v>
+      </c>
+      <c r="W12" t="s">
         <v>86</v>
       </c>
-      <c r="J12" t="s">
-        <v>242</v>
-      </c>
-      <c r="M12" t="s">
-        <v>243</v>
-      </c>
-      <c r="O12" t="s">
-        <v>244</v>
-      </c>
-      <c r="R12" t="s">
-        <v>245</v>
-      </c>
-      <c r="T12" t="s">
-        <v>246</v>
-      </c>
-      <c r="W12" t="s">
-        <v>253</v>
-      </c>
       <c r="Y12" t="s">
-        <v>254</v>
+        <v>211</v>
       </c>
       <c r="BF12" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI12" t="s">
+        <v>168</v>
+      </c>
+      <c r="BL12" t="s">
+        <v>212</v>
+      </c>
+      <c r="BO12" t="s">
+        <v>221</v>
+      </c>
+      <c r="BR12" t="s">
         <v>213</v>
-      </c>
-      <c r="BI12" t="s">
-        <v>214</v>
-      </c>
-      <c r="BL12" t="s">
-        <v>255</v>
-      </c>
-      <c r="BO12" t="s">
-        <v>256</v>
-      </c>
-      <c r="BR12" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C13" t="s">
-        <v>110</v>
-      </c>
-      <c r="E13">
-        <v>4</v>
-      </c>
-      <c r="H13" t="s">
-        <v>258</v>
-      </c>
-      <c r="J13" t="s">
-        <v>259</v>
-      </c>
-      <c r="M13" t="s">
-        <v>243</v>
-      </c>
-      <c r="O13" t="s">
-        <v>244</v>
-      </c>
-      <c r="R13" t="s">
-        <v>245</v>
-      </c>
-      <c r="T13" t="s">
-        <v>246</v>
-      </c>
-      <c r="W13" t="s">
-        <v>86</v>
-      </c>
-      <c r="Y13" t="s">
-        <v>260</v>
-      </c>
-      <c r="BF13" t="s">
-        <v>213</v>
-      </c>
-      <c r="BI13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
+      <c r="BL13" t="s">
         <v>214</v>
-      </c>
-      <c r="BL13" t="s">
-        <v>261</v>
-      </c>
-      <c r="BO13" t="s">
-        <v>270</v>
-      </c>
-      <c r="BR13" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="14" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D14" s="2"/>
+      <c r="C14" t="s">
+        <v>113</v>
+      </c>
       <c r="E14" s="2">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="H14" t="s">
+        <v>215</v>
+      </c>
+      <c r="J14" t="s">
+        <v>216</v>
+      </c>
+      <c r="M14" t="s">
+        <v>217</v>
+      </c>
+      <c r="O14" t="s">
+        <v>218</v>
+      </c>
+      <c r="BF14" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI14" t="s">
+        <v>219</v>
       </c>
       <c r="BL14" t="s">
-        <v>263</v>
+        <v>220</v>
+      </c>
+      <c r="BO14" t="s">
+        <v>222</v>
+      </c>
+      <c r="BR14" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="15" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B15" s="1"/>
+        <v>112</v>
+      </c>
       <c r="C15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E15" s="2">
         <v>2</v>
       </c>
       <c r="H15" t="s">
-        <v>264</v>
+        <v>215</v>
       </c>
       <c r="J15" t="s">
-        <v>265</v>
+        <v>224</v>
       </c>
       <c r="M15" t="s">
-        <v>266</v>
+        <v>217</v>
       </c>
       <c r="O15" t="s">
-        <v>267</v>
+        <v>225</v>
       </c>
       <c r="BF15" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI15" t="s">
-        <v>268</v>
+        <v>219</v>
       </c>
       <c r="BL15" t="s">
-        <v>269</v>
+        <v>226</v>
       </c>
       <c r="BO15" t="s">
-        <v>271</v>
+        <v>227</v>
       </c>
       <c r="BR15" t="s">
-        <v>272</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C16" t="s">
-        <v>116</v>
-      </c>
-      <c r="E16" s="2">
-        <v>2</v>
+        <v>121</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
       </c>
       <c r="H16" t="s">
-        <v>264</v>
-      </c>
-      <c r="J16" t="s">
-        <v>273</v>
-      </c>
-      <c r="M16" t="s">
-        <v>266</v>
-      </c>
-      <c r="O16" t="s">
-        <v>274</v>
+        <v>215</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>229</v>
       </c>
       <c r="BF16" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI16" t="s">
-        <v>268</v>
+        <v>219</v>
       </c>
       <c r="BL16" t="s">
-        <v>275</v>
+        <v>230</v>
       </c>
       <c r="BO16" t="s">
-        <v>276</v>
+        <v>231</v>
       </c>
       <c r="BR16" t="s">
-        <v>277</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C17" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E17">
-        <v>1</v>
-      </c>
-      <c r="H17" t="s">
-        <v>264</v>
-      </c>
-      <c r="J17" t="s">
-        <v>278</v>
+        <v>0</v>
       </c>
       <c r="BF17" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="BI17" t="s">
-        <v>268</v>
+        <v>233</v>
       </c>
       <c r="BL17" t="s">
-        <v>279</v>
+        <v>234</v>
       </c>
       <c r="BO17" t="s">
-        <v>280</v>
+        <v>235</v>
       </c>
       <c r="BR17" t="s">
-        <v>281</v>
+        <v>236</v>
       </c>
     </row>
     <row r="18" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C18" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E18">
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>264</v>
+        <v>86</v>
       </c>
       <c r="J18" t="s">
-        <v>278</v>
+        <v>237</v>
       </c>
       <c r="BF18" t="s">
-        <v>213</v>
+        <v>86</v>
       </c>
       <c r="BI18" t="s">
-        <v>268</v>
+        <v>238</v>
       </c>
       <c r="BL18" t="s">
-        <v>282</v>
+        <v>239</v>
       </c>
       <c r="BO18" t="s">
-        <v>283</v>
+        <v>240</v>
       </c>
       <c r="BR18" t="s">
-        <v>284</v>
+        <v>241</v>
       </c>
     </row>
     <row r="19" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>121</v>
+      <c r="A19" s="4" t="s">
+        <v>118</v>
       </c>
       <c r="C19" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="H19" t="s">
-        <v>264</v>
+        <v>86</v>
       </c>
       <c r="J19" t="s">
-        <v>285</v>
+        <v>243</v>
       </c>
       <c r="BF19" t="s">
-        <v>86</v>
+        <v>196</v>
       </c>
       <c r="BI19" t="s">
-        <v>286</v>
+        <v>242</v>
       </c>
       <c r="BL19" t="s">
-        <v>287</v>
+        <v>244</v>
       </c>
       <c r="BO19" t="s">
-        <v>288</v>
+        <v>245</v>
       </c>
       <c r="BR19" t="s">
-        <v>289</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>123</v>
+      <c r="A20" t="s">
+        <v>119</v>
       </c>
       <c r="C20" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
-      <c r="H20" t="s">
-        <v>264</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="BF20" t="s">
-        <v>213</v>
-      </c>
-      <c r="BI20" t="s">
-        <v>268</v>
-      </c>
-      <c r="BL20" t="s">
-        <v>290</v>
-      </c>
-      <c r="BO20" t="s">
-        <v>291</v>
-      </c>
-      <c r="BR20" t="s">
-        <v>292</v>
-      </c>
     </row>
     <row r="21" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
-        <v>125</v>
+      <c r="A21" t="s">
+        <v>120</v>
       </c>
       <c r="C21" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
-      <c r="H21" t="s">
-        <v>264</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="BF21" t="s">
-        <v>213</v>
-      </c>
-      <c r="BI21" t="s">
-        <v>268</v>
-      </c>
-      <c r="BL21" t="s">
-        <v>294</v>
-      </c>
-      <c r="BO21" t="s">
-        <v>295</v>
-      </c>
-      <c r="BR21" t="s">
-        <v>296</v>
-      </c>
     </row>
     <row r="22" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>127</v>
+      <c r="A22" t="s">
+        <v>122</v>
       </c>
       <c r="C22" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:70" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" t="s">
+        <v>135</v>
+      </c>
+      <c r="E23">
         <v>0</v>
       </c>
-      <c r="BF22" t="s">
-        <v>213</v>
-      </c>
-      <c r="BI22" t="s">
-        <v>297</v>
-      </c>
-      <c r="BL22" t="s">
-        <v>298</v>
-      </c>
-      <c r="BO22" t="s">
-        <v>299</v>
-      </c>
-      <c r="BR22" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="23" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C23" t="s">
-        <v>130</v>
-      </c>
-      <c r="E23">
-        <v>1</v>
-      </c>
-      <c r="H23" t="s">
-        <v>86</v>
-      </c>
-      <c r="J23" t="s">
-        <v>301</v>
-      </c>
-      <c r="BF23" t="s">
-        <v>86</v>
-      </c>
-      <c r="BI23" t="s">
-        <v>302</v>
-      </c>
-      <c r="BL23" t="s">
-        <v>303</v>
-      </c>
-      <c r="BO23" t="s">
-        <v>304</v>
-      </c>
-      <c r="BR23" t="s">
-        <v>305</v>
-      </c>
     </row>
     <row r="24" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A24" s="5" t="s">
-        <v>131</v>
+      <c r="A24" t="s">
+        <v>126</v>
       </c>
       <c r="C24" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="E24">
-        <v>1</v>
-      </c>
-      <c r="H24" t="s">
-        <v>86</v>
-      </c>
-      <c r="J24" t="s">
-        <v>307</v>
-      </c>
-      <c r="BF24" t="s">
-        <v>245</v>
-      </c>
-      <c r="BI24" t="s">
-        <v>306</v>
-      </c>
-      <c r="BL24" t="s">
-        <v>308</v>
-      </c>
-      <c r="BO24" t="s">
-        <v>309</v>
-      </c>
-      <c r="BR24" t="s">
-        <v>310</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C25" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2677,21 +2372,21 @@
     </row>
     <row r="26" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C26" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C27" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2699,496 +2394,243 @@
     </row>
     <row r="28" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C28" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C29" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C30" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C31" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C32" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="C33" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="E33">
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="C34" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="C35" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E35">
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="C36" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E36">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="C37" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E37">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="C38" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E38">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="C39" t="s">
         <v>162</v>
       </c>
       <c r="E39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>163</v>
+        <v>268</v>
       </c>
       <c r="C40" t="s">
-        <v>164</v>
+        <v>247</v>
       </c>
       <c r="E40">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="BF40" t="s">
+        <v>194</v>
+      </c>
+      <c r="BI40" t="s">
+        <v>251</v>
+      </c>
+      <c r="BL40" t="s">
+        <v>252</v>
+      </c>
+      <c r="BO40" t="s">
+        <v>253</v>
+      </c>
+      <c r="BR40" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="41" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>165</v>
+        <v>269</v>
       </c>
       <c r="C41" t="s">
-        <v>166</v>
+        <v>248</v>
       </c>
       <c r="E41">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="BF41" t="s">
+        <v>194</v>
+      </c>
+      <c r="BI41" t="s">
+        <v>255</v>
+      </c>
+      <c r="BL41" t="s">
+        <v>256</v>
+      </c>
+      <c r="BO41" t="s">
+        <v>257</v>
+      </c>
+      <c r="BR41" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="42" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>167</v>
+        <v>270</v>
       </c>
       <c r="C42" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="E42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="BF42" t="s">
+        <v>259</v>
+      </c>
+      <c r="BI42" t="s">
+        <v>260</v>
+      </c>
+      <c r="BL42" t="s">
+        <v>261</v>
+      </c>
+      <c r="BO42" t="s">
+        <v>265</v>
+      </c>
+      <c r="BR42" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="43" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>169</v>
+        <v>271</v>
       </c>
       <c r="C43" t="s">
-        <v>170</v>
+        <v>250</v>
       </c>
       <c r="E43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>171</v>
-      </c>
-      <c r="C44" t="s">
-        <v>172</v>
-      </c>
-      <c r="E44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>173</v>
-      </c>
-      <c r="C45" t="s">
-        <v>174</v>
-      </c>
-      <c r="E45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>175</v>
-      </c>
-      <c r="C46" t="s">
-        <v>176</v>
-      </c>
-      <c r="E46">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>177</v>
-      </c>
-      <c r="C47" t="s">
-        <v>178</v>
-      </c>
-      <c r="E47">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>179</v>
-      </c>
-      <c r="C48" t="s">
-        <v>180</v>
-      </c>
-      <c r="E48">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>181</v>
-      </c>
-      <c r="C49" t="s">
-        <v>182</v>
-      </c>
-      <c r="E49">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>183</v>
-      </c>
-      <c r="C50" t="s">
-        <v>184</v>
-      </c>
-      <c r="E50">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>185</v>
-      </c>
-      <c r="C51" t="s">
-        <v>186</v>
-      </c>
-      <c r="E51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>187</v>
-      </c>
-      <c r="C52" t="s">
-        <v>188</v>
-      </c>
-      <c r="E52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>189</v>
-      </c>
-      <c r="C53" t="s">
-        <v>190</v>
-      </c>
-      <c r="E53">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>191</v>
-      </c>
-      <c r="C54" t="s">
-        <v>192</v>
-      </c>
-      <c r="E54">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>193</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="BF43" t="s">
         <v>194</v>
       </c>
-      <c r="E55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>195</v>
-      </c>
-      <c r="C56" t="s">
-        <v>196</v>
-      </c>
-      <c r="E56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>197</v>
-      </c>
-      <c r="C57" t="s">
-        <v>198</v>
-      </c>
-      <c r="E57">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>199</v>
-      </c>
-      <c r="C58" t="s">
-        <v>200</v>
-      </c>
-      <c r="E58">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>201</v>
-      </c>
-      <c r="C59" t="s">
-        <v>202</v>
-      </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>203</v>
-      </c>
-      <c r="C60" t="s">
-        <v>204</v>
-      </c>
-      <c r="E60">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="61" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>205</v>
-      </c>
-      <c r="C61" t="s">
-        <v>206</v>
-      </c>
-      <c r="E61">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>207</v>
-      </c>
-      <c r="C62" t="s">
-        <v>208</v>
-      </c>
-      <c r="E62">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>311</v>
-      </c>
-      <c r="C63" t="s">
-        <v>315</v>
-      </c>
-      <c r="E63">
-        <v>0</v>
-      </c>
-      <c r="BF63" t="s">
-        <v>243</v>
-      </c>
-      <c r="BI63" t="s">
-        <v>319</v>
-      </c>
-      <c r="BL63" t="s">
-        <v>320</v>
-      </c>
-      <c r="BO63" t="s">
-        <v>321</v>
-      </c>
-      <c r="BR63" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="64" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>312</v>
-      </c>
-      <c r="C64" t="s">
-        <v>316</v>
-      </c>
-      <c r="E64">
-        <v>0</v>
-      </c>
-      <c r="BF64" t="s">
-        <v>243</v>
-      </c>
-      <c r="BI64" t="s">
-        <v>323</v>
-      </c>
-      <c r="BL64" t="s">
-        <v>324</v>
-      </c>
-      <c r="BO64" t="s">
-        <v>325</v>
-      </c>
-      <c r="BR64" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="65" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>313</v>
-      </c>
-      <c r="C65" t="s">
-        <v>317</v>
-      </c>
-      <c r="E65">
-        <v>0</v>
-      </c>
-      <c r="BF65" t="s">
-        <v>327</v>
-      </c>
-      <c r="BI65" t="s">
-        <v>328</v>
-      </c>
-      <c r="BL65" t="s">
-        <v>329</v>
-      </c>
-      <c r="BO65" t="s">
-        <v>333</v>
-      </c>
-      <c r="BR65" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="66" spans="1:70" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>314</v>
-      </c>
-      <c r="C66" t="s">
-        <v>318</v>
-      </c>
-      <c r="E66">
-        <v>0</v>
-      </c>
-      <c r="BF66" t="s">
-        <v>243</v>
-      </c>
-      <c r="BI66" t="s">
-        <v>331</v>
-      </c>
-      <c r="BL66" t="s">
-        <v>332</v>
-      </c>
-      <c r="BO66" t="s">
-        <v>335</v>
-      </c>
-      <c r="BR66" t="s">
-        <v>334</v>
+      <c r="BI43" t="s">
+        <v>263</v>
+      </c>
+      <c r="BL43" t="s">
+        <v>264</v>
+      </c>
+      <c r="BO43" t="s">
+        <v>267</v>
+      </c>
+      <c r="BR43" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J21" r:id="rId1" display="Sally@EmuSoftware.Com" xr:uid="{89E1025F-7416-854B-BFAE-C980E993CAED}"/>
+    <hyperlink ref="J16" r:id="rId1" display="Sally@EmuSoftware.Com" xr:uid="{89E1025F-7416-854B-BFAE-C980E993CAED}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update: Added all required info to the testing script.
I added all the info to the testing script.  This made sure it worked as intended.
</commit_message>
<xml_diff>
--- a/Test-Cases/Testing-Script-Records.xlsx
+++ b/Test-Cases/Testing-Script-Records.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexahope/Documents/GitHub/Ophelias-Oasis/Test-Cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8457345-59F6-F145-9DA9-1EB50F273981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B472E466-5119-5240-878D-145B646F3A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" firstSheet="1" activeTab="1" xr2:uid="{32C5AFC3-1601-AE47-BE56-3877807D3FAA}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="335">
   <si>
     <t>Transaction ID:</t>
   </si>
@@ -804,9 +804,6 @@
     <t xml:space="preserve">The are no parameters for this function.  A local entry in the database changes those entries.  </t>
   </si>
   <si>
-    <t>The output is a integer state how many days you must book in advanced.  You must change those entries for the data it's self to change.</t>
-  </si>
-  <si>
     <t>5, 10, 15, 20, 25, 30, 35, 40, 45, 50</t>
   </si>
   <si>
@@ -856,6 +853,198 @@
   </si>
   <si>
     <t>Function 42:</t>
+  </si>
+  <si>
+    <t>Sam, Bern, Keith, Harvey, Sam, Drake, Eithan, Lee, Nick, Jack</t>
+  </si>
+  <si>
+    <t>"Report that this user has been acting not well.  The user is not doing anything to help us as a people.  We need to work together as a pople to make sure we can understand why this user is acting this way", "Good bed", "Sad night", "Old shoes", "Hard night.", "Sad job.", "Bad person.", "Old life.", "Nice day on the beach.", "Had a rought day in high school."</t>
+  </si>
+  <si>
+    <t>The function create a new report and store it in the mainframe.</t>
+  </si>
+  <si>
+    <t>The two parameters are the name of the person and the description of the report.</t>
+  </si>
+  <si>
+    <t>The function output true when the report has been saved and false when the report save has failed.</t>
+  </si>
+  <si>
+    <t>"Long report.", "Older report of the website.", "A new report.", "A old system report.", "A newer system report.", "Different system report.", "Code report changed due to old system of management.", "Newer system of management.", "Used system of management.", "Changing to reflect present demographic."</t>
+  </si>
+  <si>
+    <t>The function will make sure to modify a report on a person.  It will do so by managing the report and changing it based on the needs of the person.</t>
+  </si>
+  <si>
+    <t>The two parameters are the name of the person the report is on and the report itself.</t>
+  </si>
+  <si>
+    <t>The function will output a true if the users report correct was changed and otherwise it will output a false.</t>
+  </si>
+  <si>
+    <t>This function will delete a report from a user by name.  Then it will make sure the user does not see the report again.</t>
+  </si>
+  <si>
+    <t>The parameter is the name of the user who's report we are trying to delete.</t>
+  </si>
+  <si>
+    <t>The function outputs true when the update was successful and the user report was deleted.  Otherwise, it will report false when this does not occur.</t>
+  </si>
+  <si>
+    <t>The function will display the logo.</t>
+  </si>
+  <si>
+    <t>Their are no parameters.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function outputs true when the logo is displayed.  It will output false when the logo is not displayed.  </t>
+  </si>
+  <si>
+    <t>[12, 4, 2014], [9, 7, 2020], [11, 8, 2020], [2, 13, 2026], [7, 19, 2026], [4, 31, 2026], [7, 23, 2026], [9, 25, 2026], [5, 17, 2025], [9, 14, 19]</t>
+  </si>
+  <si>
+    <t>There are two parameters.  The first is the name of the booking user.  The secton is th e date of the modify booking value.</t>
+  </si>
+  <si>
+    <t>The function will output true when the booking has been modify and false otherwise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function is for modifying the booking reports.  It double check what the booking report is and modifys it accoding to what is required for the booking report.  </t>
+  </si>
+  <si>
+    <t>The function is for deleting a booking report.  It will be used to delete a booking report by name.</t>
+  </si>
+  <si>
+    <t>There is one parameter which is the name of the user whos booking report we are deleting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The function will output true when the booking report is deleted.  It will output false when the booking report was not deleted.  </t>
+  </si>
+  <si>
+    <t>"The Lost See", "The user activity book", "Lost on ice", "Using the project as a guild.", "Looking for places to hid.", "Looking for the program requirments.", "Looking for the project working as intended.", "Making sure the project is working as intended.", "Double checking the project looks how it should.", "Modifying the project to make sure it works as intended."</t>
+  </si>
+  <si>
+    <t>String[3], String[1], String[2], String[5], String[1], String[8], String[2], String[3], String[3], String[3]</t>
+  </si>
+  <si>
+    <t>["Hiya", "Mo", "Mu"], ["Laya"], ["Rama", "Gama"], ["Maya", "Mo", "Mu", "Taya", "Maya"], ["Maya"], ["Maya", "Tim", "Lue", "Tris", "Leo", "Nardo", "Kim", "Kriss"], ["Kim", "Kriss"], ["Canna", "Skip", "Autume"], ["Rita", "Pita", "Tristin"], ["Lossifiticion", "Nositritial", "Nerficica"]</t>
+  </si>
+  <si>
+    <t>The function uses the names of users to make sure to construct a project report.  The project uses the project report value and the names of the user to construct a project report.</t>
+  </si>
+  <si>
+    <t>There are two parameters that are being used.  The first one is the name of the project report.  The second one is the names of the users involved in the project report.</t>
+  </si>
+  <si>
+    <t>The output for the function is true when the project output is correct.  It is false when the project output is false.</t>
+  </si>
+  <si>
+    <t>"The Lost See", "The user activity book", "Lost on ice", "Using the project as a guild.", "Looking for places to hid.", "Looking for the program requirments.", "Looking for the project working as intended.", "Making sure the project is working as intended</t>
+  </si>
+  <si>
+    <t>The function is used to view the project report.</t>
+  </si>
+  <si>
+    <t>There is one parameter which is the name of the project report.</t>
+  </si>
+  <si>
+    <t>The output is true when the operation is successful and false otherwise.</t>
+  </si>
+  <si>
+    <t>The function deletes the project report.</t>
+  </si>
+  <si>
+    <t>Their is one parameter which si the name of the project report.</t>
+  </si>
+  <si>
+    <t>"The update report.", "New report.", "Old report.", "Lost report.", "Used report.", "Using new report.", "Using old report.", "Using lost report.", "Using lost stolen.", "Using newer report structure."</t>
+  </si>
+  <si>
+    <t>The function changes the current report.  It allows for a custom report to be created.</t>
+  </si>
+  <si>
+    <t>There are three parameters, the user name, date, and, new report string.</t>
+  </si>
+  <si>
+    <t>"Room 1", "Room 2", "Room 3", "Room 4", "Room 5", "Room 6", "Room 7", "Room 8", "Room 9", "Room 10"</t>
+  </si>
+  <si>
+    <t>The function for report a new transaction as it occurs.  This can include rooms being reserved.</t>
+  </si>
+  <si>
+    <t>There is one parameter which includes a description of the latest transaction.  This allows for the user to understand the transaction.</t>
+  </si>
+  <si>
+    <t>The function creates a new transaction with the users name for the transaction and the description of the transaction.</t>
+  </si>
+  <si>
+    <t>There are two parameters.  The first one is for the name of the user.  The second is for the description of the transaction.</t>
+  </si>
+  <si>
+    <t>There is one parameter which is the description of the transaction.</t>
+  </si>
+  <si>
+    <t>The function delete the new transaction by description.</t>
+  </si>
+  <si>
+    <t>"Room 2", "Room 3", "Room 5", "Room 7", "Room 8", "Room 9", "Room 10", "Room 11", "Room 8", "Room 9"</t>
+  </si>
+  <si>
+    <t>The function modifies the existing transaction.  It changes it so the transaction looks different based on the name of the users transaction.</t>
+  </si>
+  <si>
+    <t>There is two parameters.  The first is for the name of the user.  The second is for the transaction description.</t>
+  </si>
+  <si>
+    <t>"Uploads/New-file-1.img", "Uploads/New-file-2.img", "Uploads/New-file-3.img", "Uploads/New-file-4.img", "Uploads/New-file-5.img", "Uploads/New-file-6.img", "Uploads/New-file-7.img", "Uploads/New-file-8.img", "Uploads/New-file-9.img", "Uploads/New-file-10.img"</t>
+  </si>
+  <si>
+    <t>The function is their for modifying the user profile image.  It can modify the current user profile image.</t>
+  </si>
+  <si>
+    <t>There are two parameters.  The first one is the one for modifying the user profile by name.  The second on is the the one for using the new file for changing the contents of the user profile.</t>
+  </si>
+  <si>
+    <t>The function deletes user profile.</t>
+  </si>
+  <si>
+    <t>The parameter is the name of the user who is being deleated.</t>
+  </si>
+  <si>
+    <t>The function displays a confirmation code for the users involed.</t>
+  </si>
+  <si>
+    <t>The parameter is the name of the user for the confirmation code.</t>
+  </si>
+  <si>
+    <t>The function will minimize the user QR code.  This will allow for the user not the see the QR code.</t>
+  </si>
+  <si>
+    <t>Their is no parameters involved.</t>
+  </si>
+  <si>
+    <t>Sam, Ben, Keith, Harvey, Sam, Drake, Eithan, Lee, Nick, Jack</t>
+  </si>
+  <si>
+    <t>This function is for delating the report reservtion.  This is required for making sure all entries are relvant.</t>
+  </si>
+  <si>
+    <t>There is one parameter for the name of the user who's entry we are deleting.</t>
+  </si>
+  <si>
+    <t>Double, Double, Double, Double, Double, Double, Double, Double, Double, Double</t>
+  </si>
+  <si>
+    <t>20.31, 21,44, 51.93, 57.66, 58.99, 41.88, 55.41, 57.32, 88.91, 41.57</t>
+  </si>
+  <si>
+    <t>The function is for adding the report reservation pricing.  It add the reservation pricing by user name.</t>
+  </si>
+  <si>
+    <t>There are two parameters.  One is for user name which state the name of the user booking.  The other is for the parameters fo the booking process.</t>
+  </si>
+  <si>
+    <t>The output is the number of days which is in the form of a interger.</t>
   </si>
 </sst>
 </file>
@@ -2312,7 +2501,34 @@
         <v>129</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="H20" t="s">
+        <v>86</v>
+      </c>
+      <c r="J20" t="s">
+        <v>271</v>
+      </c>
+      <c r="M20" t="s">
+        <v>86</v>
+      </c>
+      <c r="O20" t="s">
+        <v>272</v>
+      </c>
+      <c r="BF20" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI20" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL20" t="s">
+        <v>273</v>
+      </c>
+      <c r="BO20" t="s">
+        <v>274</v>
+      </c>
+      <c r="BR20" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:70" x14ac:dyDescent="0.2">
@@ -2323,7 +2539,34 @@
         <v>131</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="H21" t="s">
+        <v>86</v>
+      </c>
+      <c r="J21" t="s">
+        <v>271</v>
+      </c>
+      <c r="M21" t="s">
+        <v>86</v>
+      </c>
+      <c r="O21" t="s">
+        <v>276</v>
+      </c>
+      <c r="BF21" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI21" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL21" t="s">
+        <v>277</v>
+      </c>
+      <c r="BO21" t="s">
+        <v>278</v>
+      </c>
+      <c r="BR21" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="22" spans="1:70" x14ac:dyDescent="0.2">
@@ -2336,6 +2579,27 @@
       <c r="E22">
         <v>1</v>
       </c>
+      <c r="H22" t="s">
+        <v>86</v>
+      </c>
+      <c r="J22" t="s">
+        <v>271</v>
+      </c>
+      <c r="BF22" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI22" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL22" t="s">
+        <v>280</v>
+      </c>
+      <c r="BO22" t="s">
+        <v>281</v>
+      </c>
+      <c r="BR22" t="s">
+        <v>282</v>
+      </c>
     </row>
     <row r="23" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
@@ -2347,6 +2611,21 @@
       <c r="E23">
         <v>0</v>
       </c>
+      <c r="BF23" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI23" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL23" t="s">
+        <v>283</v>
+      </c>
+      <c r="BO23" t="s">
+        <v>284</v>
+      </c>
+      <c r="BR23" t="s">
+        <v>285</v>
+      </c>
     </row>
     <row r="24" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
@@ -2358,6 +2637,33 @@
       <c r="E24">
         <v>2</v>
       </c>
+      <c r="H24" t="s">
+        <v>86</v>
+      </c>
+      <c r="J24" t="s">
+        <v>271</v>
+      </c>
+      <c r="M24" t="s">
+        <v>196</v>
+      </c>
+      <c r="O24" t="s">
+        <v>286</v>
+      </c>
+      <c r="BF24" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI24" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL24" t="s">
+        <v>289</v>
+      </c>
+      <c r="BO24" t="s">
+        <v>287</v>
+      </c>
+      <c r="BR24" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="25" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
@@ -2369,6 +2675,27 @@
       <c r="E25">
         <v>1</v>
       </c>
+      <c r="H25" t="s">
+        <v>86</v>
+      </c>
+      <c r="J25" t="s">
+        <v>271</v>
+      </c>
+      <c r="BF25" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI25" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL25" t="s">
+        <v>290</v>
+      </c>
+      <c r="BO25" t="s">
+        <v>291</v>
+      </c>
+      <c r="BR25" t="s">
+        <v>292</v>
+      </c>
     </row>
     <row r="26" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
@@ -2380,6 +2707,33 @@
       <c r="E26">
         <v>2</v>
       </c>
+      <c r="H26" t="s">
+        <v>86</v>
+      </c>
+      <c r="J26" t="s">
+        <v>293</v>
+      </c>
+      <c r="M26" t="s">
+        <v>294</v>
+      </c>
+      <c r="O26" t="s">
+        <v>295</v>
+      </c>
+      <c r="BF26" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI26" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL26" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="BO26" t="s">
+        <v>297</v>
+      </c>
+      <c r="BR26" t="s">
+        <v>298</v>
+      </c>
     </row>
     <row r="27" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
@@ -2391,6 +2745,27 @@
       <c r="E27">
         <v>1</v>
       </c>
+      <c r="H27" t="s">
+        <v>86</v>
+      </c>
+      <c r="J27" t="s">
+        <v>299</v>
+      </c>
+      <c r="BF27" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI27" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL27" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="BO27" t="s">
+        <v>301</v>
+      </c>
+      <c r="BR27" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="28" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
@@ -2400,7 +2775,28 @@
         <v>149</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="H28" t="s">
+        <v>86</v>
+      </c>
+      <c r="J28" t="s">
+        <v>299</v>
+      </c>
+      <c r="BF28" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI28" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL28" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="BO28" t="s">
+        <v>304</v>
+      </c>
+      <c r="BR28" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="29" spans="1:70" x14ac:dyDescent="0.2">
@@ -2413,6 +2809,39 @@
       <c r="E29">
         <v>3</v>
       </c>
+      <c r="H29" t="s">
+        <v>86</v>
+      </c>
+      <c r="J29" t="s">
+        <v>299</v>
+      </c>
+      <c r="M29" t="s">
+        <v>196</v>
+      </c>
+      <c r="O29" t="s">
+        <v>286</v>
+      </c>
+      <c r="R29" t="s">
+        <v>86</v>
+      </c>
+      <c r="T29" t="s">
+        <v>305</v>
+      </c>
+      <c r="BF29" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI29" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL29" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="BO29" t="s">
+        <v>307</v>
+      </c>
+      <c r="BR29" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="30" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
@@ -2424,6 +2853,27 @@
       <c r="E30">
         <v>1</v>
       </c>
+      <c r="H30" t="s">
+        <v>86</v>
+      </c>
+      <c r="J30" t="s">
+        <v>308</v>
+      </c>
+      <c r="BF30" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI30" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL30" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="BO30" t="s">
+        <v>310</v>
+      </c>
+      <c r="BR30" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="31" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
@@ -2435,6 +2885,33 @@
       <c r="E31">
         <v>2</v>
       </c>
+      <c r="H31" t="s">
+        <v>86</v>
+      </c>
+      <c r="J31" t="s">
+        <v>271</v>
+      </c>
+      <c r="M31" t="s">
+        <v>86</v>
+      </c>
+      <c r="O31" t="s">
+        <v>308</v>
+      </c>
+      <c r="BF31" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI31" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL31" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="BO31" t="s">
+        <v>312</v>
+      </c>
+      <c r="BR31" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="32" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
@@ -2446,6 +2923,27 @@
       <c r="E32">
         <v>1</v>
       </c>
+      <c r="H32" t="s">
+        <v>86</v>
+      </c>
+      <c r="J32" t="s">
+        <v>308</v>
+      </c>
+      <c r="BF32" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI32" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL32" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="BO32" t="s">
+        <v>313</v>
+      </c>
+      <c r="BR32" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="33" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
@@ -2457,6 +2955,33 @@
       <c r="E33">
         <v>2</v>
       </c>
+      <c r="H33" t="s">
+        <v>86</v>
+      </c>
+      <c r="J33" t="s">
+        <v>271</v>
+      </c>
+      <c r="M33" t="s">
+        <v>86</v>
+      </c>
+      <c r="O33" t="s">
+        <v>315</v>
+      </c>
+      <c r="BF33" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI33" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL33" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="BO33" t="s">
+        <v>317</v>
+      </c>
+      <c r="BR33" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="34" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
@@ -2468,6 +2993,33 @@
       <c r="E34">
         <v>2</v>
       </c>
+      <c r="H34" t="s">
+        <v>86</v>
+      </c>
+      <c r="J34" t="s">
+        <v>271</v>
+      </c>
+      <c r="M34" t="s">
+        <v>86</v>
+      </c>
+      <c r="O34" t="s">
+        <v>318</v>
+      </c>
+      <c r="BF34" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI34" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL34" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="BO34" t="s">
+        <v>320</v>
+      </c>
+      <c r="BR34" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="35" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
@@ -2477,7 +3029,28 @@
         <v>158</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="H35" t="s">
+        <v>86</v>
+      </c>
+      <c r="J35" t="s">
+        <v>271</v>
+      </c>
+      <c r="BF35" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI35" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL35" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="BO35" t="s">
+        <v>322</v>
+      </c>
+      <c r="BR35" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="36" spans="1:70" x14ac:dyDescent="0.2">
@@ -2490,6 +3063,27 @@
       <c r="E36">
         <v>1</v>
       </c>
+      <c r="H36" t="s">
+        <v>86</v>
+      </c>
+      <c r="J36" t="s">
+        <v>271</v>
+      </c>
+      <c r="BF36" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI36" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL36" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="BO36" t="s">
+        <v>324</v>
+      </c>
+      <c r="BR36" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="37" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
@@ -2501,6 +3095,21 @@
       <c r="E37">
         <v>0</v>
       </c>
+      <c r="BF37" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI37" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL37" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="BO37" t="s">
+        <v>326</v>
+      </c>
+      <c r="BR37" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="38" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
@@ -2512,6 +3121,27 @@
       <c r="E38">
         <v>1</v>
       </c>
+      <c r="H38" t="s">
+        <v>86</v>
+      </c>
+      <c r="J38" t="s">
+        <v>327</v>
+      </c>
+      <c r="BF38" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI38" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL38" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="BO38" t="s">
+        <v>329</v>
+      </c>
+      <c r="BR38" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="39" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
@@ -2523,10 +3153,37 @@
       <c r="E39">
         <v>2</v>
       </c>
+      <c r="H39" t="s">
+        <v>86</v>
+      </c>
+      <c r="J39" t="s">
+        <v>327</v>
+      </c>
+      <c r="M39" t="s">
+        <v>330</v>
+      </c>
+      <c r="O39" t="s">
+        <v>331</v>
+      </c>
+      <c r="BF39" t="s">
+        <v>167</v>
+      </c>
+      <c r="BI39" t="s">
+        <v>219</v>
+      </c>
+      <c r="BL39" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="BO39" t="s">
+        <v>333</v>
+      </c>
+      <c r="BR39" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="40" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C40" t="s">
         <v>247</v>
@@ -2547,12 +3204,12 @@
         <v>253</v>
       </c>
       <c r="BR40" t="s">
-        <v>254</v>
+        <v>334</v>
       </c>
     </row>
     <row r="41" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C41" t="s">
         <v>248</v>
@@ -2564,21 +3221,21 @@
         <v>194</v>
       </c>
       <c r="BI41" t="s">
+        <v>254</v>
+      </c>
+      <c r="BL41" t="s">
         <v>255</v>
       </c>
-      <c r="BL41" t="s">
+      <c r="BO41" t="s">
         <v>256</v>
       </c>
-      <c r="BO41" t="s">
+      <c r="BR41" t="s">
         <v>257</v>
-      </c>
-      <c r="BR41" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C42" t="s">
         <v>249</v>
@@ -2587,24 +3244,24 @@
         <v>0</v>
       </c>
       <c r="BF42" t="s">
+        <v>258</v>
+      </c>
+      <c r="BI42" t="s">
         <v>259</v>
       </c>
-      <c r="BI42" t="s">
+      <c r="BL42" t="s">
         <v>260</v>
       </c>
-      <c r="BL42" t="s">
+      <c r="BO42" t="s">
+        <v>264</v>
+      </c>
+      <c r="BR42" t="s">
         <v>261</v>
-      </c>
-      <c r="BO42" t="s">
-        <v>265</v>
-      </c>
-      <c r="BR42" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="43" spans="1:70" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C43" t="s">
         <v>250</v>
@@ -2616,16 +3273,16 @@
         <v>194</v>
       </c>
       <c r="BI43" t="s">
+        <v>262</v>
+      </c>
+      <c r="BL43" t="s">
         <v>263</v>
       </c>
-      <c r="BL43" t="s">
-        <v>264</v>
-      </c>
       <c r="BO43" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="BR43" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>